<commit_message>
Update missing-spec sheet: add brand-website lookup column
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bi-led-thieu-lens-cong-suat-2026-10-15.xlsx
+++ b/docs/bi-led-thieu-lens-cong-suat-2026-10-15.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="101">
   <si>
     <t>STT</t>
   </si>
@@ -50,6 +50,9 @@
     <t>Pha cần nhập (W)</t>
   </si>
   <si>
+    <t>Gợi ý từ website hãng (cần đối chiếu)</t>
+  </si>
+  <si>
     <t>Người nhập</t>
   </si>
   <si>
@@ -77,6 +80,9 @@
     <t>Có: Cos ~55W Cos/bi / Pha ~90W Pha/bi</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>Henvvei</t>
   </si>
   <si>
@@ -101,7 +107,7 @@
     <t>Có: 3.0 inch</t>
   </si>
   <si>
-    <t/>
+    <t>Lens 3.0 Inch · Cos 45W · Pha 55W — https://titanmoto.vn/bi-led-titan-moto-cb750</t>
   </si>
   <si>
     <t>X-Light</t>
@@ -114,6 +120,9 @@
   </si>
   <si>
     <t>Có: Cos 55W / Pha 65W</t>
+  </si>
+  <si>
+    <t>Cos 55W (mô tả) · Pha 65W (mô tả) — https://x-light.vn/bi-led-x-light-x5-pro</t>
   </si>
   <si>
     <t>GTR</t>
@@ -714,7 +723,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:O30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -728,11 +737,12 @@
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="12" width="15" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="24" customWidth="1"/>
+    <col min="13" max="13" width="46" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -775,995 +785,1085 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E2" s="2">
         <v>9000000</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I2" s="5"/>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
+      <c r="M2" t="s">
+        <v>22</v>
+      </c>
       <c r="N2" s="5"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O2" s="5"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E3" s="2">
         <v>8000000</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
+      <c r="M3" t="s">
+        <v>22</v>
+      </c>
       <c r="N3" s="5"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O3" s="5"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E4" s="2">
         <v>7000000</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H4" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="I4" s="5"/>
       <c r="J4" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K4" s="5"/>
       <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
+      <c r="M4" t="s">
+        <v>31</v>
+      </c>
       <c r="N4" s="5"/>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O4" s="5"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5" s="2">
         <v>8500000</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
+      <c r="M5" t="s">
+        <v>36</v>
+      </c>
       <c r="N5" s="5"/>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O5" s="5"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H6" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
+      <c r="M6" t="s">
+        <v>22</v>
+      </c>
       <c r="N6" s="5"/>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O6" s="5"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I7" s="5"/>
       <c r="J7" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
+      <c r="M7" t="s">
+        <v>22</v>
+      </c>
       <c r="N7" s="5"/>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O7" s="5"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
+      <c r="M8" t="s">
+        <v>22</v>
+      </c>
       <c r="N8" s="5"/>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O8" s="5"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H9" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K9" s="5"/>
       <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
+      <c r="M9" t="s">
+        <v>22</v>
+      </c>
       <c r="N9" s="5"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O9" s="5"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E10" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I10" s="5"/>
       <c r="J10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
+      <c r="M10" t="s">
+        <v>22</v>
+      </c>
       <c r="N10" s="5"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O10" s="5"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I11" s="5"/>
       <c r="J11" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
+      <c r="M11" t="s">
+        <v>22</v>
+      </c>
       <c r="N11" s="5"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O11" s="5"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I12" s="5"/>
       <c r="J12" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
+      <c r="M12" t="s">
+        <v>22</v>
+      </c>
       <c r="N12" s="5"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O12" s="5"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E13" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I13" s="5"/>
       <c r="J13" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
+      <c r="M13" t="s">
+        <v>22</v>
+      </c>
       <c r="N13" s="5"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O13" s="5"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E14" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H14" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I14" s="5"/>
       <c r="J14" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
+      <c r="M14" t="s">
+        <v>22</v>
+      </c>
       <c r="N14" s="5"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O14" s="5"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H15" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I15" s="5"/>
       <c r="J15" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
+      <c r="M15" t="s">
+        <v>22</v>
+      </c>
       <c r="N15" s="5"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O15" s="5"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I16" s="5"/>
       <c r="J16" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
+      <c r="M16" t="s">
+        <v>22</v>
+      </c>
       <c r="N16" s="5"/>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O16" s="5"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E17" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H17" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I17" s="5"/>
       <c r="J17" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
+      <c r="M17" t="s">
+        <v>22</v>
+      </c>
       <c r="N17" s="5"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O17" s="5"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D18" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I18" s="5"/>
       <c r="J18" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
+      <c r="M18" t="s">
+        <v>22</v>
+      </c>
       <c r="N18" s="5"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O18" s="5"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D19" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E19" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H19" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I19" s="5"/>
       <c r="J19" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
+      <c r="M19" t="s">
+        <v>22</v>
+      </c>
       <c r="N19" s="5"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O19" s="5"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C20" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D20" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E20" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H20" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I20" s="5"/>
       <c r="J20" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
+      <c r="M20" t="s">
+        <v>22</v>
+      </c>
       <c r="N20" s="5"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O20" s="5"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D21" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E21" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H21" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I21" s="5"/>
       <c r="J21" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
+      <c r="M21" t="s">
+        <v>22</v>
+      </c>
       <c r="N21" s="5"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O21" s="5"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C22" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D22" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E22" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H22" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I22" s="5"/>
       <c r="J22" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
+      <c r="M22" t="s">
+        <v>22</v>
+      </c>
       <c r="N22" s="5"/>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O22" s="5"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D23" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E23" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H23" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I23" s="5"/>
       <c r="J23" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
+      <c r="M23" t="s">
+        <v>22</v>
+      </c>
       <c r="N23" s="5"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O23" s="5"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24" t="s">
+        <v>39</v>
+      </c>
+      <c r="E24" t="s">
+        <v>40</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="G24" t="s">
         <v>30</v>
       </c>
-      <c r="C24" t="s">
-        <v>79</v>
-      </c>
-      <c r="D24" t="s">
-        <v>36</v>
-      </c>
-      <c r="E24" t="s">
-        <v>37</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G24" t="s">
-        <v>28</v>
-      </c>
       <c r="H24" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="I24" s="5"/>
       <c r="J24" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
+      <c r="M24" t="s">
+        <v>22</v>
+      </c>
       <c r="N24" s="5"/>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O24" s="5"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D25" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E25" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I25" s="5"/>
       <c r="J25" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
+      <c r="M25" t="s">
+        <v>22</v>
+      </c>
       <c r="N25" s="5"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O25" s="5"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D26" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E26" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H26" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I26" s="5"/>
       <c r="J26" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
+      <c r="M26" t="s">
+        <v>22</v>
+      </c>
       <c r="N26" s="5"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O26" s="5"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D27" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E27" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H27" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I27" s="5"/>
       <c r="J27" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K27" s="5"/>
       <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
+      <c r="M27" t="s">
+        <v>22</v>
+      </c>
       <c r="N27" s="5"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O27" s="5"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D28" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E28" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H28" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K28" s="5"/>
       <c r="L28" s="5"/>
-      <c r="M28" s="5"/>
+      <c r="M28" t="s">
+        <v>22</v>
+      </c>
       <c r="N28" s="5"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O28" s="5"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C29" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D29" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E29" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H29" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I29" s="5"/>
       <c r="J29" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K29" s="5"/>
       <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
+      <c r="M29" t="s">
+        <v>22</v>
+      </c>
       <c r="N29" s="5"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O29" s="5"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C30" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D30" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E30" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H30" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I30" s="5"/>
       <c r="J30" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K30" s="5"/>
       <c r="L30" s="5"/>
-      <c r="M30" s="5"/>
+      <c r="M30" t="s">
+        <v>22</v>
+      </c>
       <c r="N30" s="5"/>
+      <c r="O30" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1"/>
+  <autoFilter ref="A1:O1"/>
   <hyperlinks>
     <hyperlink ref="F2" r:id="rId1"/>
     <hyperlink ref="F3" r:id="rId2"/>
@@ -1810,27 +1910,27 @@
   <sheetData>
     <row r="1" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:1" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>